<commit_message>
cleaned up the workflow
</commit_message>
<xml_diff>
--- a/data/raw/ica_extraction_master_with_notes.xlsx
+++ b/data/raw/ica_extraction_master_with_notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timsc\Documents\GitHub\ica-methods-synthesis\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A69021-3651-4215-885F-AA5A3A9BC1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649DEEA9-C98A-4F25-91B9-92CFB10C5C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{252201E6-B0A3-4A6F-B0C8-EDC2E224CCCA}"/>
   </bookViews>
@@ -3972,7 +3972,7 @@
         <v>25</v>
       </c>
       <c r="BP4" t="s">
-        <v>32</v>
+        <v>360</v>
       </c>
       <c r="BQ4" t="b">
         <v>0</v>
@@ -4253,7 +4253,7 @@
         <v>201</v>
       </c>
       <c r="BP5" t="s">
-        <v>32</v>
+        <v>360</v>
       </c>
       <c r="BQ5" t="b">
         <v>0</v>
@@ -4537,7 +4537,7 @@
         <v>169</v>
       </c>
       <c r="BP6" t="s">
-        <v>32</v>
+        <v>360</v>
       </c>
       <c r="BQ6" t="b">
         <v>0</v>
@@ -5093,7 +5093,7 @@
         <v>222</v>
       </c>
       <c r="BP8" t="s">
-        <v>32</v>
+        <v>360</v>
       </c>
       <c r="BQ8" t="b">
         <v>0</v>
@@ -6220,7 +6220,7 @@
         <v>25</v>
       </c>
       <c r="BP12" t="s">
-        <v>32</v>
+        <v>360</v>
       </c>
       <c r="BQ12" t="b">
         <v>0</v>
@@ -7691,7 +7691,7 @@
         <v>572</v>
       </c>
       <c r="CP17" t="s">
-        <v>360</v>
+        <v>758</v>
       </c>
       <c r="CQ17" t="s">
         <v>758</v>
@@ -8253,7 +8253,7 @@
         <v>573</v>
       </c>
       <c r="CP19" t="s">
-        <v>360</v>
+        <v>758</v>
       </c>
       <c r="CQ19" t="s">
         <v>758</v>
@@ -11607,10 +11607,10 @@
         <v>407</v>
       </c>
       <c r="CP31" t="s">
-        <v>360</v>
+        <v>758</v>
       </c>
       <c r="CQ31" t="s">
-        <v>360</v>
+        <v>758</v>
       </c>
     </row>
     <row r="32" spans="1:97">

</xml_diff>